<commit_message>
ASTA: MLUX and SSZX replaced by X
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/ASTA_Index_Current.xlsx
+++ b/src/sastadev/data/methods/ASTA_Index_Current.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CACDC261-39AA-43BF-A77B-999A06D62FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC561DCB-DBCF-4A04-88C4-DF1AD3A315B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -722,9 +722,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -762,7 +762,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -868,7 +868,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1010,7 +1010,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1794,10 +1794,10 @@
         <v>27</v>
       </c>
       <c r="E28" t="s">
+        <v>28</v>
+      </c>
+      <c r="F28" t="s">
         <v>198</v>
-      </c>
-      <c r="F28" t="s">
-        <v>28</v>
       </c>
       <c r="H28" t="s">
         <v>15</v>
@@ -2160,10 +2160,10 @@
         <v>16</v>
       </c>
       <c r="E43" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F43" s="4" t="s">
         <v>199</v>
-      </c>
-      <c r="F43" t="s">
-        <v>28</v>
       </c>
       <c r="H43" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
comm_noncom + Bepaler weg version 1
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/ASTA_Index_Current.xlsx
+++ b/src/sastadev/data/methods/ASTA_Index_Current.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC561DCB-DBCF-4A04-88C4-DF1AD3A315B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7433EB40-A015-4867-96C4-0E764A0C6E70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="202">
   <si>
     <t>ID</t>
   </si>
@@ -263,9 +263,6 @@
     <t xml:space="preserve"> substitutie van een lidwoord</t>
   </si>
   <si>
-    <t xml:space="preserve"> deletie van een lidwoord</t>
-  </si>
-  <si>
     <t xml:space="preserve"> deletie subject</t>
   </si>
   <si>
@@ -639,6 +636,12 @@
   </si>
   <si>
     <t>//node[@pt="ww" and %ASTA_modalww% and not(%ASTA_XXX%)]</t>
+  </si>
+  <si>
+    <t>get_missing_det</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> deletie van een lidwoord;tijdelijk uitgezet</t>
   </si>
 </sst>
 </file>
@@ -722,9 +725,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -762,7 +765,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -868,7 +871,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1010,7 +1013,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1062,31 +1065,31 @@
         <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="P1" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>186</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>11</v>
@@ -1105,28 +1108,28 @@
         <v>31</v>
       </c>
       <c r="F2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H2" t="s">
         <v>15</v>
       </c>
       <c r="I2" t="s">
+        <v>134</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="L2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N2" t="s">
+        <v>129</v>
+      </c>
+      <c r="R2" t="s">
+        <v>196</v>
+      </c>
+      <c r="U2" t="s">
         <v>135</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="L2" t="s">
-        <v>15</v>
-      </c>
-      <c r="N2" t="s">
-        <v>130</v>
-      </c>
-      <c r="R2" t="s">
-        <v>197</v>
-      </c>
-      <c r="U2" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.3">
@@ -1149,7 +1152,7 @@
         <v>15</v>
       </c>
       <c r="N3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.3">
@@ -1172,13 +1175,13 @@
         <v>12</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L4" t="s">
         <v>15</v>
       </c>
       <c r="N4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U4" t="s">
         <v>40</v>
@@ -1192,10 +1195,10 @@
         <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H5" t="s">
         <v>15</v>
@@ -1207,7 +1210,7 @@
         <v>15</v>
       </c>
       <c r="N5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.3">
@@ -1218,10 +1221,10 @@
         <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H6" t="s">
         <v>15</v>
@@ -1233,7 +1236,7 @@
         <v>15</v>
       </c>
       <c r="N6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.3">
@@ -1241,14 +1244,14 @@
         <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E7" t="s">
+        <v>103</v>
+      </c>
+      <c r="F7" t="s">
         <v>104</v>
       </c>
-      <c r="F7" t="s">
-        <v>105</v>
-      </c>
       <c r="H7" t="s">
         <v>15</v>
       </c>
@@ -1256,7 +1259,7 @@
         <v>15</v>
       </c>
       <c r="N7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U7" t="s">
         <v>70</v>
@@ -1282,7 +1285,7 @@
         <v>15</v>
       </c>
       <c r="N8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.3">
@@ -1296,19 +1299,19 @@
         <v>25</v>
       </c>
       <c r="F9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H9" t="s">
         <v>15</v>
       </c>
       <c r="K9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L9" t="s">
         <v>15</v>
       </c>
       <c r="N9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.3">
@@ -1319,25 +1322,25 @@
         <v>18</v>
       </c>
       <c r="E10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F10" t="s">
         <v>117</v>
       </c>
-      <c r="F10" t="s">
-        <v>118</v>
-      </c>
       <c r="H10" t="s">
         <v>15</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L10" t="s">
         <v>15</v>
       </c>
       <c r="N10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U10" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.3">
@@ -1360,7 +1363,7 @@
         <v>15</v>
       </c>
       <c r="N11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.3">
@@ -1383,7 +1386,7 @@
         <v>15</v>
       </c>
       <c r="N12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.3">
@@ -1406,7 +1409,7 @@
         <v>15</v>
       </c>
       <c r="N13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.3">
@@ -1420,7 +1423,7 @@
         <v>29</v>
       </c>
       <c r="F14" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H14" t="s">
         <v>15</v>
@@ -1429,16 +1432,16 @@
         <v>37</v>
       </c>
       <c r="K14" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="L14" t="s">
         <v>15</v>
       </c>
       <c r="N14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="Q14" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="U14" t="s">
         <v>38</v>
@@ -1452,10 +1455,10 @@
         <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H15" t="s">
         <v>15</v>
@@ -1464,7 +1467,7 @@
         <v>15</v>
       </c>
       <c r="N15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.3">
@@ -1472,13 +1475,13 @@
         <v>54</v>
       </c>
       <c r="D16" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E16" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H16" t="s">
         <v>15</v>
@@ -1487,7 +1490,7 @@
         <v>15</v>
       </c>
       <c r="N16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.3">
@@ -1495,13 +1498,13 @@
         <v>55</v>
       </c>
       <c r="D17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E17" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H17" t="s">
         <v>15</v>
@@ -1510,7 +1513,7 @@
         <v>15</v>
       </c>
       <c r="N17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
@@ -1518,14 +1521,14 @@
         <v>56</v>
       </c>
       <c r="D18" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E18" t="s">
+        <v>105</v>
+      </c>
+      <c r="F18" t="s">
         <v>106</v>
       </c>
-      <c r="F18" t="s">
-        <v>107</v>
-      </c>
       <c r="H18" t="s">
         <v>15</v>
       </c>
@@ -1533,7 +1536,7 @@
         <v>15</v>
       </c>
       <c r="N18" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U18" t="s">
         <v>69</v>
@@ -1556,17 +1559,17 @@
         <v>9</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M19" s="3"/>
       <c r="N19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="Q19" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="R19" s="3"/>
       <c r="S19" s="3"/>
@@ -1589,16 +1592,16 @@
         <v>15</v>
       </c>
       <c r="K20" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="L20" t="s">
         <v>15</v>
       </c>
       <c r="N20" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="Q20" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.3">
@@ -1618,19 +1621,19 @@
         <v>8</v>
       </c>
       <c r="K21" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L21" t="s">
         <v>15</v>
       </c>
       <c r="N21" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="Q21" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="U21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.3">
@@ -1641,10 +1644,10 @@
         <v>18</v>
       </c>
       <c r="E22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F22" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H22" t="s">
         <v>15</v>
@@ -1653,16 +1656,16 @@
         <v>10</v>
       </c>
       <c r="K22" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="L22" t="s">
         <v>15</v>
       </c>
       <c r="N22" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="Q22" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.3">
@@ -1688,7 +1691,7 @@
         <v>15</v>
       </c>
       <c r="N23" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.3">
@@ -1705,13 +1708,13 @@
         <v>37</v>
       </c>
       <c r="L24" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="N24" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U24" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.3">
@@ -1725,19 +1728,19 @@
         <v>26</v>
       </c>
       <c r="F25" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H25" t="s">
         <v>15</v>
       </c>
       <c r="K25" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="L25" t="s">
         <v>15</v>
       </c>
       <c r="N25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.3">
@@ -1754,13 +1757,13 @@
         <v>37</v>
       </c>
       <c r="L26" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="N26" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U26" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.3">
@@ -1783,7 +1786,7 @@
         <v>15</v>
       </c>
       <c r="N27" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.3">
@@ -1797,19 +1800,19 @@
         <v>28</v>
       </c>
       <c r="F28" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H28" t="s">
         <v>15</v>
       </c>
       <c r="K28" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="L28" t="s">
         <v>15</v>
       </c>
       <c r="N28" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.3">
@@ -1820,7 +1823,7 @@
         <v>18</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H29" t="s">
         <v>15</v>
@@ -1829,7 +1832,7 @@
         <v>15</v>
       </c>
       <c r="N29" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U29" t="s">
         <v>71</v>
@@ -1837,13 +1840,13 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D30" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H30" t="s">
         <v>15</v>
@@ -1852,7 +1855,7 @@
         <v>15</v>
       </c>
       <c r="N30" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U30" t="s">
         <v>72</v>
@@ -1860,13 +1863,13 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D31" t="s">
         <v>18</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H31" t="s">
         <v>15</v>
@@ -1875,7 +1878,7 @@
         <v>15</v>
       </c>
       <c r="N31" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U31" t="s">
         <v>73</v>
@@ -1883,16 +1886,16 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D32" t="s">
         <v>18</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F32" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H32" t="s">
         <v>15</v>
@@ -1901,7 +1904,7 @@
         <v>15</v>
       </c>
       <c r="N32" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U32" t="s">
         <v>74</v>
@@ -1909,16 +1912,16 @@
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D33" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F33" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H33" t="s">
         <v>15</v>
@@ -1927,24 +1930,27 @@
         <v>15</v>
       </c>
       <c r="N33" t="s">
-        <v>130</v>
+        <v>129</v>
+      </c>
+      <c r="T33" t="s">
+        <v>200</v>
       </c>
       <c r="U33" t="s">
-        <v>75</v>
+        <v>201</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D34" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F34" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H34" t="s">
         <v>15</v>
@@ -1953,21 +1959,21 @@
         <v>15</v>
       </c>
       <c r="N34" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D35" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H35" t="s">
         <v>15</v>
@@ -1976,21 +1982,21 @@
         <v>15</v>
       </c>
       <c r="N35" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U35" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D36" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H36" t="s">
         <v>15</v>
@@ -1999,21 +2005,21 @@
         <v>15</v>
       </c>
       <c r="N36" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D37" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H37" t="s">
         <v>15</v>
@@ -2022,139 +2028,139 @@
         <v>15</v>
       </c>
       <c r="N37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U37" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
+        <v>96</v>
+      </c>
+      <c r="D38" t="s">
+        <v>193</v>
+      </c>
+      <c r="E38" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D38" t="s">
-        <v>194</v>
-      </c>
-      <c r="E38" s="4" t="s">
+      <c r="F38" t="s">
+        <v>165</v>
+      </c>
+      <c r="H38" t="s">
+        <v>15</v>
+      </c>
+      <c r="L38" t="s">
+        <v>15</v>
+      </c>
+      <c r="N38" t="s">
+        <v>129</v>
+      </c>
+      <c r="U38" t="s">
         <v>98</v>
-      </c>
-      <c r="F38" t="s">
-        <v>166</v>
-      </c>
-      <c r="H38" t="s">
-        <v>15</v>
-      </c>
-      <c r="L38" t="s">
-        <v>15</v>
-      </c>
-      <c r="N38" t="s">
-        <v>130</v>
-      </c>
-      <c r="U38" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D39" t="s">
         <v>18</v>
       </c>
       <c r="E39" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F39" t="s">
+        <v>141</v>
+      </c>
+      <c r="H39" t="s">
         <v>119</v>
       </c>
-      <c r="F39" t="s">
-        <v>142</v>
-      </c>
-      <c r="H39" t="s">
+      <c r="L39" t="s">
+        <v>15</v>
+      </c>
+      <c r="N39" t="s">
+        <v>129</v>
+      </c>
+      <c r="U39" t="s">
         <v>120</v>
-      </c>
-      <c r="L39" t="s">
-        <v>15</v>
-      </c>
-      <c r="N39" t="s">
-        <v>130</v>
-      </c>
-      <c r="U39" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D40" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H40" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L40" t="s">
         <v>15</v>
       </c>
       <c r="N40" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U40" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D41" t="s">
         <v>18</v>
       </c>
       <c r="E41" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="H41" t="s">
+        <v>119</v>
+      </c>
+      <c r="L41" t="s">
+        <v>15</v>
+      </c>
+      <c r="N41" t="s">
+        <v>129</v>
+      </c>
+      <c r="U41" t="s">
         <v>125</v>
-      </c>
-      <c r="H41" t="s">
-        <v>120</v>
-      </c>
-      <c r="L41" t="s">
-        <v>15</v>
-      </c>
-      <c r="N41" t="s">
-        <v>130</v>
-      </c>
-      <c r="U41" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D42" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F42" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H42" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L42" t="s">
         <v>15</v>
       </c>
       <c r="N42" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U42" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D43" t="s">
         <v>16</v>
@@ -2163,178 +2169,178 @@
         <v>28</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H43" t="s">
         <v>15</v>
       </c>
       <c r="K43" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L43" t="s">
         <v>15</v>
       </c>
       <c r="N43" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
+        <v>145</v>
+      </c>
+      <c r="D44" t="s">
         <v>146</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="H44" t="s">
+        <v>15</v>
+      </c>
+      <c r="K44" t="s">
+        <v>168</v>
+      </c>
+      <c r="L44" t="s">
+        <v>15</v>
+      </c>
+      <c r="N44" t="s">
         <v>147</v>
       </c>
-      <c r="E44" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="H44" t="s">
-        <v>15</v>
-      </c>
-      <c r="K44" t="s">
-        <v>169</v>
-      </c>
-      <c r="L44" t="s">
-        <v>15</v>
-      </c>
-      <c r="N44" t="s">
-        <v>148</v>
-      </c>
       <c r="U44" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
+        <v>148</v>
+      </c>
+      <c r="D45" t="s">
         <v>149</v>
       </c>
-      <c r="D45" t="s">
+      <c r="H45" t="s">
+        <v>15</v>
+      </c>
+      <c r="K45" t="s">
         <v>150</v>
       </c>
-      <c r="H45" t="s">
-        <v>15</v>
-      </c>
-      <c r="K45" t="s">
+      <c r="L45" t="s">
+        <v>119</v>
+      </c>
+      <c r="N45" t="s">
+        <v>153</v>
+      </c>
+      <c r="U45" t="s">
         <v>151</v>
-      </c>
-      <c r="L45" t="s">
-        <v>120</v>
-      </c>
-      <c r="N45" t="s">
-        <v>154</v>
-      </c>
-      <c r="U45" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D46" t="s">
         <v>18</v>
       </c>
       <c r="E46" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="H46" t="s">
+        <v>119</v>
+      </c>
+      <c r="L46" t="s">
+        <v>119</v>
+      </c>
+      <c r="N46" t="s">
+        <v>129</v>
+      </c>
+      <c r="R46" t="s">
+        <v>186</v>
+      </c>
+      <c r="U46" t="s">
         <v>156</v>
-      </c>
-      <c r="H46" t="s">
-        <v>120</v>
-      </c>
-      <c r="L46" t="s">
-        <v>120</v>
-      </c>
-      <c r="N46" t="s">
-        <v>130</v>
-      </c>
-      <c r="R46" t="s">
-        <v>187</v>
-      </c>
-      <c r="U46" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D47" t="s">
+        <v>146</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="H47" t="s">
+        <v>15</v>
+      </c>
+      <c r="K47" t="s">
+        <v>171</v>
+      </c>
+      <c r="L47" t="s">
+        <v>119</v>
+      </c>
+      <c r="N47" t="s">
         <v>147</v>
       </c>
-      <c r="E47" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="H47" t="s">
-        <v>15</v>
-      </c>
-      <c r="K47" t="s">
-        <v>172</v>
-      </c>
-      <c r="L47" t="s">
-        <v>120</v>
-      </c>
-      <c r="N47" t="s">
-        <v>148</v>
-      </c>
       <c r="U47" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D48" t="s">
         <v>18</v>
       </c>
       <c r="E48" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="F48" t="s">
         <v>175</v>
       </c>
-      <c r="F48" t="s">
-        <v>176</v>
-      </c>
       <c r="H48" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L48" t="s">
         <v>15</v>
       </c>
       <c r="N48" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="U48" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
+        <v>187</v>
+      </c>
+      <c r="D49" t="s">
+        <v>146</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="H49" t="s">
+        <v>15</v>
+      </c>
+      <c r="K49" t="s">
+        <v>190</v>
+      </c>
+      <c r="L49" t="s">
+        <v>15</v>
+      </c>
+      <c r="N49" t="s">
+        <v>129</v>
+      </c>
+      <c r="O49" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>189</v>
+      </c>
+      <c r="U49" t="s">
         <v>188</v>
-      </c>
-      <c r="D49" t="s">
-        <v>147</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H49" t="s">
-        <v>15</v>
-      </c>
-      <c r="K49" t="s">
-        <v>191</v>
-      </c>
-      <c r="L49" t="s">
-        <v>15</v>
-      </c>
-      <c r="N49" t="s">
-        <v>130</v>
-      </c>
-      <c r="O49" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q49" t="s">
-        <v>190</v>
-      </c>
-      <c r="U49" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.3">

</xml_diff>